<commit_message>
Update daily job results
</commit_message>
<xml_diff>
--- a/data/ranked_jobs_2026-06-04.xlsx
+++ b/data/ranked_jobs_2026-06-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,16 @@
           <t>Reason</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Matched Skills</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Missing Skills</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -525,7 +535,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -534,9 +544,11 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Matched skills: .net, c#, angular, sql server, web application</t>
-        </is>
-      </c>
+          <t>AI ranking failed: 'str' object has no attribute 'choices'</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -585,18 +597,20 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Matched skills: angular, typescript, dashboard</t>
-        </is>
-      </c>
+          <t>AI ranking failed: 'str' object has no attribute 'choices'</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>